<commit_message>
Also include regular names
</commit_message>
<xml_diff>
--- a/Extra_data/flights.xlsx
+++ b/Extra_data/flights.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F230"/>
+  <dimension ref="A1:H230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,10 +446,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>origin_icao</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>destination_icao</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>destination</t>
         </is>
@@ -484,6 +494,16 @@
           <t>EGPF</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Glasgow International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -514,6 +534,16 @@
           <t>EHBK</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -544,6 +574,16 @@
           <t>EHTW</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Twente Airport</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -574,6 +614,16 @@
           <t>LEGE</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Girona-Costa Brava Airport</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -604,6 +654,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -634,6 +694,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -664,6 +734,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -694,6 +774,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Midden-Zeeland Airfield</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -724,6 +814,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -754,6 +854,16 @@
           <t>EDCS</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Genk Zwartberg Airfield</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Saarmund Airfield</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -784,6 +894,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -814,6 +934,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Düsseldorf Airport</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -844,6 +974,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>London Gatwick Airport</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -874,6 +1014,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>London City Airport</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -904,6 +1054,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Entebbe International Airport</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -934,6 +1094,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Budapest Liszt Ferenc International Airport</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -964,6 +1134,16 @@
           <t>EHBK</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -994,6 +1174,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Francisco de Sá Carneiro Airport</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1024,6 +1214,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1054,6 +1254,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1084,6 +1294,16 @@
           <t>EHLW</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Leeuwarden Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -1114,6 +1334,16 @@
           <t>EHLW</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Kleine Brogel Air Base</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Leeuwarden Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1144,6 +1374,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1174,6 +1414,16 @@
           <t>EGPH</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Edinburgh Airport</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1204,6 +1454,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Václav Havel Airport Prague</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1234,6 +1494,16 @@
           <t>EKCH</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Copenhagen Kastrup Airport</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -1264,6 +1534,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>İstanbul Atatürk Airport</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1294,6 +1574,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Francisco de Sá Carneiro Airport</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1324,6 +1614,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Brussels Airport</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1354,6 +1654,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Jomo Kenyatta International Airport</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1384,6 +1694,16 @@
           <t>EGCC</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Manchester Airport</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1414,6 +1734,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Vienna International Airport</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -1444,6 +1774,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Jomo Kenyatta International Airport</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1474,6 +1814,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>José Martí International Airport</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1504,6 +1854,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Ibiza Airport</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -1534,6 +1894,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Václav Havel Airport Prague</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -1564,6 +1934,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Hoogeveen Airfield</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -1594,6 +1974,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>East Midlands Airport</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -1624,6 +2014,16 @@
           <t>LPFR</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Faro Airport</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -1654,6 +2054,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pisa International Airport</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -1684,6 +2094,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -1714,6 +2134,16 @@
           <t>EIDW</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Dublin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -1744,6 +2174,16 @@
           <t>LFBE</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Bergerac Dordogne Périgord Airport</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -1774,6 +2214,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -1804,6 +2254,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Ibiza Airport</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -1834,6 +2294,16 @@
           <t>LTBS</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Dalaman International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -1864,6 +2334,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Kraków John Paul II International Airport</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -1894,6 +2374,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -1924,6 +2414,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -1954,6 +2454,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Kalamata Airport</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -1984,6 +2494,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Bergerac Dordogne Périgord Airport</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -2014,6 +2534,16 @@
           <t>LFLL</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Lyon Saint-Exupéry Airport</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -2044,6 +2574,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Munich Airport</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -2074,6 +2614,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -2104,6 +2654,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Toronto Lester B. Pearson International Airport</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -2134,6 +2694,16 @@
           <t>ENGM</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Oslo Airport, Gardermoen</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -2164,6 +2734,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Detroit Metropolitan Wayne County Airport</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -2194,6 +2774,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Geneva Cointrin International Airport</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -2224,6 +2814,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>London Gatwick Airport</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -2254,6 +2854,16 @@
           <t>LLBG</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Ben Gurion International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -2284,6 +2894,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Hartsfield Jackson Atlanta International Airport</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -2314,6 +2934,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Dublin Airport</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -2344,6 +2974,16 @@
           <t>EGPH</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Edinburgh Airport</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -2374,6 +3014,16 @@
           <t>EICK</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Cork Airport</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -2404,6 +3054,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Girona-Costa Brava Airport</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -2434,6 +3094,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -2464,6 +3134,16 @@
           <t>EHBK</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -2494,6 +3174,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -2524,6 +3214,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Nice-Côte d'Azur Airport</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -2554,6 +3254,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Ibiza Airport</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -2584,6 +3294,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Florence Airport, Peretola</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -2614,6 +3334,16 @@
           <t>ELLX</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Luxembourg-Findel International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -2644,6 +3374,16 @@
           <t>EGSS</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>London Stansted Airport</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -2674,6 +3414,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Málaga-Costa del Sol Airport</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -2704,6 +3454,16 @@
           <t>LBSF</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Sofia Airport</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -2734,6 +3494,16 @@
           <t>LTBA</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>İstanbul Atatürk Airport</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -2764,6 +3534,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -2794,6 +3574,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -2824,6 +3614,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Newark Liberty International Airport</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -2854,6 +3654,16 @@
           <t>KMCO</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Orlando International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -2884,6 +3694,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -2914,6 +3734,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -2944,6 +3774,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Gilze Rijen Air Base</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -2974,6 +3814,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -3004,6 +3854,16 @@
           <t>LIMC</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Milan Malpensa International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -3034,6 +3894,16 @@
           <t>ENVA</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Trondheim Airport, Værnes</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -3064,6 +3934,16 @@
           <t>EHBK</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -3094,6 +3974,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -3124,6 +4014,16 @@
           <t>EHTE</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Farnborough Airport</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Teuge Airport</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -3154,6 +4054,16 @@
           <t>ENCN</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Kristiansand Airport, Kjevik</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -3184,6 +4094,16 @@
           <t>LTAI</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -3214,6 +4134,16 @@
           <t>EHLW</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Leeuwarden Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -3244,6 +4174,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -3274,6 +4214,16 @@
           <t>EHTW</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Twente Airport</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -3304,6 +4254,16 @@
           <t>EGPD</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Aberdeen Dyce Airport</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -3334,6 +4294,16 @@
           <t>LEMG</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Málaga-Costa del Sol Airport</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -3364,6 +4334,16 @@
           <t>LDSP</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Split Airport</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -3394,6 +4374,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Milan Malpensa International Airport</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -3424,6 +4414,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Málaga-Costa del Sol Airport</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -3454,6 +4454,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Bergen Airport, Flesland</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -3484,6 +4494,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Aalborg Airport</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -3514,6 +4534,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -3544,6 +4574,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -3574,6 +4614,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -3604,6 +4654,16 @@
           <t>EGBB</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Birmingham Airport</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -3634,6 +4694,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Humberto Delgado Airport (Lisbon Portela Airport)</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -3664,6 +4734,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -3694,6 +4774,16 @@
           <t>EGCC</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Manchester Airport</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -3724,6 +4814,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -3754,6 +4854,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Humberto Delgado Airport (Lisbon Portela Airport)</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -3784,6 +4894,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -3814,6 +4934,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Jomo Kenyatta International Airport</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -3844,6 +4974,16 @@
           <t>ENZV</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Stavanger Airport, Sola</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -3874,6 +5014,16 @@
           <t>LTAI</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -3904,6 +5054,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Josep Tarradellas Barcelona-El Prat Airport</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -3934,6 +5094,16 @@
           <t>LROP</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Bucharest Henri Coandă International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -3964,6 +5134,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>London Luton Airport</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -3994,6 +5174,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -4024,6 +5214,16 @@
           <t>EDDV</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Hannover Airport</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -4054,6 +5254,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -4084,6 +5294,16 @@
           <t>LOWW</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Vienna International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -4114,6 +5334,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -4144,6 +5374,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -4174,6 +5414,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Seattle–Tacoma International Airport</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -4204,6 +5454,16 @@
           <t>LPPT</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Humberto Delgado Airport (Lisbon Portela Airport)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -4234,6 +5494,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>John F Kennedy International Airport</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -4264,6 +5534,16 @@
           <t>LEMG</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Málaga-Costa del Sol Airport</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -4294,6 +5574,16 @@
           <t>EDDF</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Frankfurt Airport</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -4324,6 +5614,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -4354,6 +5654,16 @@
           <t>KSLC</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Salt Lake City International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -4384,6 +5694,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -4414,6 +5734,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Stockholm-Arlanda Airport</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -4444,6 +5774,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Nantes Atlantique Airport</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -4474,6 +5814,16 @@
           <t>KDTW</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Detroit Metropolitan Wayne County Airport</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -4504,6 +5854,16 @@
           <t>EPGD</t>
         </is>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Gdańsk Lech Wałęsa Airport</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -4534,6 +5894,16 @@
           <t>EIDW</t>
         </is>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Dublin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -4564,6 +5934,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -4594,6 +5974,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Milan Malpensa International Airport</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -4624,6 +6014,16 @@
           <t>ESSA</t>
         </is>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Stockholm-Arlanda Airport</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -4654,6 +6054,16 @@
           <t>ESSL</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Linköping City Airport</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -4684,6 +6094,16 @@
           <t>LFML</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Marseille Provence Airport</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -4714,6 +6134,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Southampton Airport</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -4744,6 +6174,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -4774,6 +6214,16 @@
           <t>LEMG</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Málaga-Costa del Sol Airport</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -4804,6 +6254,16 @@
           <t>LGKO</t>
         </is>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Kos Airport</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -4834,6 +6294,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Vienna International Airport</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -4864,6 +6334,16 @@
           <t>LPFR</t>
         </is>
       </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Faro Airport</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -4894,6 +6374,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -4924,6 +6414,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -4954,6 +6454,16 @@
           <t>LGTS</t>
         </is>
       </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Thessaloniki Macedonia International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -4984,6 +6494,16 @@
           <t>EDDT</t>
         </is>
       </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Berlin-Tegel Otto Lilienthal Airport</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -5014,6 +6534,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -5044,6 +6574,16 @@
           <t>LIRF</t>
         </is>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Rome–Fiumicino Leonardo da Vinci International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -5074,6 +6614,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -5104,6 +6654,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Belfast International Airport</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -5134,6 +6694,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Birmingham Airport</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -5164,6 +6734,16 @@
           <t>LEVC</t>
         </is>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Valencia Airport</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -5194,6 +6774,16 @@
           <t>EFHK</t>
         </is>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Helsinki Vantaa Airport</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -5224,6 +6814,16 @@
           <t>EDDM</t>
         </is>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Munich Airport</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -5254,6 +6854,16 @@
           <t>EIDW</t>
         </is>
       </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Dublin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -5284,6 +6894,16 @@
           <t>EHEH</t>
         </is>
       </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>M. R. Štefánik Airport</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -5314,6 +6934,16 @@
           <t>LOWW</t>
         </is>
       </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Vienna International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -5344,6 +6974,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Jomo Kenyatta International Airport</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -5374,6 +7014,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -5404,6 +7054,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -5434,6 +7094,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -5464,6 +7134,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Stuttgart Airport</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -5494,6 +7174,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -5524,6 +7214,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -5554,6 +7254,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -5584,6 +7294,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -5614,6 +7334,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Bergen Airport, Flesland</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -5644,6 +7374,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -5674,6 +7414,16 @@
           <t>UMMS</t>
         </is>
       </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -5704,6 +7454,16 @@
           <t>EPWA</t>
         </is>
       </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Warsaw Chopin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -5734,6 +7494,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -5764,6 +7534,16 @@
           <t>SMJP</t>
         </is>
       </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -5794,6 +7574,16 @@
           <t>EGLC</t>
         </is>
       </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>London City Airport</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -5824,6 +7614,16 @@
           <t>LTAI</t>
         </is>
       </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -5854,6 +7654,16 @@
           <t>LGKF</t>
         </is>
       </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Kefallinia Airport</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -5884,6 +7694,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -5914,6 +7734,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -5944,6 +7774,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Aalborg Airport</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -5974,6 +7814,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Václav Havel Airport Prague</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -6004,6 +7854,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -6034,6 +7894,16 @@
           <t>LFPG</t>
         </is>
       </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Charles de Gaulle International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -6064,6 +7934,16 @@
           <t>EDDK</t>
         </is>
       </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Cologne Bonn Airport</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -6094,6 +7974,16 @@
           <t>LEBB</t>
         </is>
       </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Bilbao Airport</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -6124,6 +8014,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Bergen Airport, Flesland</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -6154,6 +8054,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -6184,6 +8094,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -6214,6 +8134,16 @@
           <t>EHLE</t>
         </is>
       </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Milan Bergamo Airport / Antonio Locatelli Air Base</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -6244,6 +8174,16 @@
           <t>EFHK</t>
         </is>
       </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Helsinki Vantaa Airport</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -6274,6 +8214,16 @@
           <t>LGIR</t>
         </is>
       </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Heraklion International Nikos Kazantzakis Airport</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -6304,6 +8254,16 @@
           <t>LIML</t>
         </is>
       </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Milano Linate Airport</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -6334,6 +8294,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -6364,6 +8334,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Humberto Delgado Airport (Lisbon Portela Airport)</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
@@ -6394,6 +8374,16 @@
           <t>EHGG</t>
         </is>
       </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Antalya International Airport</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Groningen Airport Eelde</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -6424,6 +8414,16 @@
           <t>EHBK</t>
         </is>
       </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Stockholm-Bromma Airport</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Maastricht Aachen Airport</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -6454,6 +8454,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -6484,6 +8494,16 @@
           <t>EGGD</t>
         </is>
       </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Bristol Airport</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -6514,6 +8534,16 @@
           <t>EBAW</t>
         </is>
       </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Antwerp International Airport (Deurne)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -6544,6 +8574,16 @@
           <t>LEBL</t>
         </is>
       </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Josep Tarradellas Barcelona-El Prat Airport</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -6574,6 +8614,16 @@
           <t>EGLC</t>
         </is>
       </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>London City Airport</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -6604,6 +8654,16 @@
           <t>EDDK</t>
         </is>
       </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Cologne Bonn Airport</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -6634,6 +8694,16 @@
           <t>EIDW</t>
         </is>
       </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Dublin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
@@ -6664,6 +8734,16 @@
           <t>EYKA</t>
         </is>
       </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Eindhoven Airport</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Kaunas International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
@@ -6694,6 +8774,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Santorini Airport</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
@@ -6724,6 +8814,16 @@
           <t>LICC</t>
         </is>
       </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Catania-Fontanarossa Airport</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
@@ -6754,6 +8854,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
@@ -6784,6 +8894,16 @@
           <t>EPWA</t>
         </is>
       </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Warsaw Chopin Airport</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
@@ -6814,6 +8934,16 @@
           <t>EHRD</t>
         </is>
       </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Rome–Fiumicino Leonardo da Vinci International Airport</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
@@ -6844,6 +8974,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Ostrava Leos Janáček Airport</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -6874,6 +9014,16 @@
           <t>EHKD</t>
         </is>
       </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Lelystad Airport</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>De Kooy Airfield / Den Helder Naval Air Station</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
@@ -6904,6 +9054,16 @@
           <t>EHLW</t>
         </is>
       </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Leeuwarden Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
@@ -6934,6 +9094,16 @@
           <t>LSGG</t>
         </is>
       </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Geneva Cointrin International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
@@ -6964,6 +9134,16 @@
           <t>LDSP</t>
         </is>
       </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Split Airport</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
@@ -6994,6 +9174,16 @@
           <t>LSZH</t>
         </is>
       </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Zürich Airport</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -7024,6 +9214,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Vienna International Airport</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
@@ -7054,6 +9254,16 @@
           <t>EGKK</t>
         </is>
       </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>London Gatwick Airport</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -7084,6 +9294,16 @@
           <t>EGLC</t>
         </is>
       </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>London City Airport</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -7114,6 +9334,16 @@
           <t>EHLW</t>
         </is>
       </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Leeuwarden Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
@@ -7144,6 +9374,16 @@
           <t>LIEO</t>
         </is>
       </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>Olbia Costa Smeralda Airport</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -7174,6 +9414,16 @@
           <t>Coordinate</t>
         </is>
       </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
@@ -7204,6 +9454,16 @@
           <t>EHAM</t>
         </is>
       </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Rome–Fiumicino Leonardo da Vinci International Airport</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
@@ -7234,6 +9494,16 @@
           <t>EVRA</t>
         </is>
       </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>Riga International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
@@ -7264,6 +9534,16 @@
           <t>EHVK</t>
         </is>
       </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>Volkel Air Base</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
@@ -7294,6 +9574,16 @@
           <t>KIAD</t>
         </is>
       </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Rotterdam The Hague Airport</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>Washington Dulles International Airport</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
@@ -7322,6 +9612,16 @@
       <c r="F230" t="inlineStr">
         <is>
           <t>SBFZ</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Amsterdam Airport Schiphol</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>Coordinate</t>
         </is>
       </c>
     </row>

</xml_diff>